<commit_message>
recreating typo to show wimp object is idenitcal to sample
</commit_message>
<xml_diff>
--- a/inst/extdata/example.wimp.xlsx
+++ b/inst/extdata/example.wimp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markheckmann/Workspace/db/WimpTools/dev/review/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markheckmann/Workspace/db/WimpTools/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF25196F-2F46-C040-89AE-BE1587A84C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB208C7-244C-5449-B874-897E95E69F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,7 +67,7 @@
     <t>Ideal-Self</t>
   </si>
   <si>
-    <t>Anxious</t>
+    <t>Ansioux</t>
   </si>
 </sst>
 </file>

</xml_diff>